<commit_message>
chore(audit): registrar auditoria da VPS de 19/10 e liquidacao de 17/10 no worklog
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-17.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-17.xlsx
@@ -578,15 +578,19 @@
       <c r="K2" t="n">
         <v>1.32</v>
       </c>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -660,15 +664,19 @@
       <c r="K3" t="n">
         <v>1.29</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>AO Away Win</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -742,15 +750,19 @@
       <c r="K4" t="n">
         <v>1.36</v>
       </c>
-      <c r="L4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -824,15 +836,19 @@
       <c r="K5" t="n">
         <v>1.33</v>
       </c>
-      <c r="L5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>RED</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">

</xml_diff>

<commit_message>
feat(forward): consolidar 8 jogos de 17/10 a tarde no ledger e na planilha oficial
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-17.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-17.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -872,6 +872,694 @@
       </c>
       <c r="T5" t="n">
         <v>34.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ukrainian Premier League</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Shakhtar x Kolos Kovalyovka</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Shakhtar</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Kolos Kovalyovka</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>230</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>200</v>
+      </c>
+      <c r="S6" t="n">
+        <v>34.48</v>
+      </c>
+      <c r="T6" t="n">
+        <v>32.76</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>French Ligue 1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Strasbourg x Paris St-G</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Strasbourg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Paris St-G</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>2730</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>200</v>
+      </c>
+      <c r="S7" t="n">
+        <v>31.25</v>
+      </c>
+      <c r="T7" t="n">
+        <v>29.69</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Italian Serie A</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Bologna x Inter</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Bologna</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Inter</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>1421</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>200</v>
+      </c>
+      <c r="S8" t="n">
+        <v>34.48</v>
+      </c>
+      <c r="T8" t="n">
+        <v>32.76</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Turkish Super League</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Fenerbahce x Alanyaspor</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Fenerbahce</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Alanyaspor</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>1568</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>200</v>
+      </c>
+      <c r="S9" t="n">
+        <v>34.48</v>
+      </c>
+      <c r="T9" t="n">
+        <v>32.76</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Norwegian Eliteserien</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Viking x Fredrikstad</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Viking</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Fredrikstad</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>1628</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>200</v>
+      </c>
+      <c r="S10" t="n">
+        <v>38.46</v>
+      </c>
+      <c r="T10" t="n">
+        <v>36.54</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Spanish La Liga</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Betis x Barcelona</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Betis</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>AO Away Win</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>438</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>200</v>
+      </c>
+      <c r="S11" t="n">
+        <v>38.46</v>
+      </c>
+      <c r="T11" t="n">
+        <v>36.54</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Israeli Premier League</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Maccabi Petach Tikva x Maccabi Haifa</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Maccabi Petach Tikva</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Maccabi Haifa</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Lay Home/DC X2 (FavVis &lt;= 1.65)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>486</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>200</v>
+      </c>
+      <c r="S12" t="n">
+        <v>29.41</v>
+      </c>
+      <c r="T12" t="n">
+        <v>27.94</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dutch Eredivisie</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SC Telstar x Feyenoord</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SC Telstar</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Feyenoord</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>AO Away Win</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>✅ LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>1706</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>200</v>
+      </c>
+      <c r="S13" t="n">
+        <v>38.46</v>
+      </c>
+      <c r="T13" t="n">
+        <v>36.54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>